<commit_message>
fix template excel, fix upload excel
</commit_message>
<xml_diff>
--- a/public/download/template.xlsx
+++ b/public/download/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\I5\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Laravel\Sertifikasi-IVFI\public\download\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B159B71A-59E9-4A38-8AE5-D0EA9A67473E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC63250C-F304-48DE-B2EC-BA44DEDD993B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>nama_lengkap</t>
   </si>
@@ -49,22 +49,13 @@
     <t>Andi Saputra</t>
   </si>
   <si>
-    <t>1234567890</t>
-  </si>
-  <si>
     <t>Jakarta</t>
   </si>
   <si>
-    <t>1995-05-10</t>
-  </si>
-  <si>
     <t>L</t>
   </si>
   <si>
     <t>Jl. Merdeka No. 1</t>
-  </si>
-  <si>
-    <t>081234567890</t>
   </si>
   <si>
     <t>andi@email.com</t>
@@ -126,11 +117,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -149,9 +142,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -189,9 +182,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -224,26 +217,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -276,26 +252,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -470,19 +429,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.77734375" customWidth="1"/>
-    <col min="2" max="2" width="20.6640625" customWidth="1"/>
-    <col min="3" max="3" width="20.33203125" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
-    <col min="5" max="5" width="19.77734375" customWidth="1"/>
-    <col min="6" max="6" width="24.88671875" customWidth="1"/>
-    <col min="7" max="7" width="26.21875" customWidth="1"/>
-    <col min="8" max="8" width="35.33203125" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
+    <col min="6" max="6" width="24.85546875" customWidth="1"/>
+    <col min="7" max="7" width="26.28515625" customWidth="1"/>
+    <col min="8" max="8" width="35.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -508,30 +467,30 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2">
+        <v>1234567890</v>
+      </c>
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="3">
+        <v>34829</v>
+      </c>
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" s="2">
+        <v>6281234567890</v>
+      </c>
+      <c r="H2" t="s">
         <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix layout, title, upload excel
</commit_message>
<xml_diff>
--- a/public/download/template.xlsx
+++ b/public/download/template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Laravel\Sertifikasi-IVFI\public\download\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\laragon\www\Sertifikasi-IVFI\public\download\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC63250C-F304-48DE-B2EC-BA44DEDD993B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86CCEBB6-5823-4D72-9F61-3FDD32C0A02D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -117,13 +117,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -432,12 +436,12 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" style="4" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
-    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="4" max="4" width="25" style="3" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="24.85546875" customWidth="1"/>
-    <col min="7" max="7" width="26.28515625" customWidth="1"/>
+    <col min="7" max="7" width="26.28515625" style="2" customWidth="1"/>
     <col min="8" max="8" width="35.28515625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -445,13 +449,13 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -460,7 +464,7 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">

</xml_diff>

<commit_message>
fix birthdate upload excel and fix pagination use bootstrap 5
</commit_message>
<xml_diff>
--- a/public/download/template.xlsx
+++ b/public/download/template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\laragon\www\Sertifikasi-IVFI\public\download\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rakhmat Khaidir\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86CCEBB6-5823-4D72-9F61-3FDD32C0A02D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88554266-3AD4-425F-AFE0-37B03C8D5ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>nama_lengkap</t>
   </si>
@@ -59,6 +59,9 @@
   </si>
   <si>
     <t>andi@email.com</t>
+  </si>
+  <si>
+    <t>16-07-2006</t>
   </si>
 </sst>
 </file>
@@ -123,11 +126,11 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -436,9 +439,9 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
-    <col min="4" max="4" width="25" style="3" customWidth="1"/>
+    <col min="4" max="4" width="25" style="5" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="24.85546875" customWidth="1"/>
     <col min="7" max="7" width="26.28515625" style="2" customWidth="1"/>
@@ -449,13 +452,13 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -464,7 +467,7 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -476,13 +479,13 @@
         <v>8</v>
       </c>
       <c r="B2" s="2">
-        <v>1234567890</v>
+        <v>1710340560001</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3">
-        <v>34829</v>
+      <c r="D2" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>

</xml_diff>